<commit_message>
Update Exercício Gerência de Processos.xlsx
</commit_message>
<xml_diff>
--- a/Exercício Gerência de Processos.xlsx
+++ b/Exercício Gerência de Processos.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPasta_de_trabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabriel_piske\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gabriel_piske\Documents\GitHub\unisenai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D76BBB1F-BEFE-48EB-96EA-DC18155D55BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{052A445E-3E86-4B90-9091-E8F69A435013}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -356,8 +356,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -365,10 +366,9 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,521 +667,521 @@
       </c>
     </row>
     <row r="4" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="16"/>
-      <c r="D4" s="16"/>
-      <c r="E4" s="16"/>
-      <c r="F4" s="16"/>
-      <c r="G4" s="16"/>
-      <c r="H4" s="16"/>
-      <c r="I4" s="16"/>
-      <c r="J4" s="16"/>
-      <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="16"/>
-      <c r="O4" s="16"/>
-      <c r="P4" s="16"/>
-      <c r="Q4" s="16"/>
-      <c r="R4" s="16"/>
-      <c r="S4" s="16"/>
-      <c r="T4" s="16"/>
-      <c r="U4" s="16"/>
-      <c r="V4" s="16"/>
-      <c r="W4" s="16" t="s">
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="X4" s="16"/>
-      <c r="Y4" s="16"/>
-      <c r="Z4" s="16"/>
-      <c r="AA4" s="16"/>
-      <c r="AB4" s="16"/>
-      <c r="AC4" s="16"/>
-      <c r="AD4" s="16"/>
-      <c r="AE4" s="16"/>
-      <c r="AF4" s="16" t="s">
+      <c r="X4" s="20"/>
+      <c r="Y4" s="20"/>
+      <c r="Z4" s="20"/>
+      <c r="AA4" s="20"/>
+      <c r="AB4" s="20"/>
+      <c r="AC4" s="20"/>
+      <c r="AD4" s="20"/>
+      <c r="AE4" s="20"/>
+      <c r="AF4" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="AG4" s="16"/>
-      <c r="AH4" s="16"/>
-      <c r="AI4" s="16"/>
-      <c r="AJ4" s="16"/>
-      <c r="AK4" s="16"/>
-      <c r="AL4" s="16"/>
-      <c r="AM4" s="16"/>
-      <c r="AN4" s="16"/>
+      <c r="AG4" s="20"/>
+      <c r="AH4" s="20"/>
+      <c r="AI4" s="20"/>
+      <c r="AJ4" s="20"/>
+      <c r="AK4" s="20"/>
+      <c r="AL4" s="20"/>
+      <c r="AM4" s="20"/>
+      <c r="AN4" s="20"/>
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B5" s="17" t="s">
+      <c r="B5" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="17"/>
-      <c r="G5" s="17"/>
-      <c r="H5" s="17"/>
-      <c r="I5" s="17"/>
-      <c r="J5" s="17"/>
-      <c r="K5" s="17"/>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="17"/>
-      <c r="O5" s="17"/>
-      <c r="P5" s="17"/>
-      <c r="Q5" s="17"/>
-      <c r="R5" s="17"/>
-      <c r="S5" s="17"/>
-      <c r="T5" s="17"/>
-      <c r="U5" s="17"/>
-      <c r="V5" s="17"/>
-      <c r="W5" s="17">
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="18"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="18"/>
+      <c r="I5" s="18"/>
+      <c r="J5" s="18"/>
+      <c r="K5" s="18"/>
+      <c r="L5" s="18"/>
+      <c r="M5" s="18"/>
+      <c r="N5" s="18"/>
+      <c r="O5" s="18"/>
+      <c r="P5" s="18"/>
+      <c r="Q5" s="18"/>
+      <c r="R5" s="18"/>
+      <c r="S5" s="18"/>
+      <c r="T5" s="18"/>
+      <c r="U5" s="18"/>
+      <c r="V5" s="18"/>
+      <c r="W5" s="18">
         <v>13748</v>
       </c>
-      <c r="X5" s="17"/>
-      <c r="Y5" s="17"/>
-      <c r="Z5" s="17"/>
-      <c r="AA5" s="17"/>
-      <c r="AB5" s="17"/>
-      <c r="AC5" s="17"/>
-      <c r="AD5" s="17"/>
-      <c r="AE5" s="17"/>
-      <c r="AF5" s="17" t="s">
+      <c r="X5" s="18"/>
+      <c r="Y5" s="18"/>
+      <c r="Z5" s="18"/>
+      <c r="AA5" s="18"/>
+      <c r="AB5" s="18"/>
+      <c r="AC5" s="18"/>
+      <c r="AD5" s="18"/>
+      <c r="AE5" s="18"/>
+      <c r="AF5" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="AG5" s="17"/>
-      <c r="AH5" s="17"/>
-      <c r="AI5" s="17"/>
-      <c r="AJ5" s="17"/>
-      <c r="AK5" s="17"/>
-      <c r="AL5" s="17"/>
-      <c r="AM5" s="17"/>
-      <c r="AN5" s="17"/>
+      <c r="AG5" s="18"/>
+      <c r="AH5" s="18"/>
+      <c r="AI5" s="18"/>
+      <c r="AJ5" s="18"/>
+      <c r="AK5" s="18"/>
+      <c r="AL5" s="18"/>
+      <c r="AM5" s="18"/>
+      <c r="AN5" s="18"/>
     </row>
     <row r="6" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="18"/>
-      <c r="H6" s="18"/>
-      <c r="I6" s="18"/>
-      <c r="J6" s="18"/>
-      <c r="K6" s="18"/>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="18"/>
-      <c r="O6" s="18"/>
-      <c r="P6" s="18"/>
-      <c r="Q6" s="18"/>
-      <c r="R6" s="18"/>
-      <c r="S6" s="18"/>
-      <c r="T6" s="18"/>
-      <c r="U6" s="18"/>
-      <c r="V6" s="18"/>
-      <c r="W6" s="18">
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="19"/>
+      <c r="G6" s="19"/>
+      <c r="H6" s="19"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="19"/>
+      <c r="K6" s="19"/>
+      <c r="L6" s="19"/>
+      <c r="M6" s="19"/>
+      <c r="N6" s="19"/>
+      <c r="O6" s="19"/>
+      <c r="P6" s="19"/>
+      <c r="Q6" s="19"/>
+      <c r="R6" s="19"/>
+      <c r="S6" s="19"/>
+      <c r="T6" s="19"/>
+      <c r="U6" s="19"/>
+      <c r="V6" s="19"/>
+      <c r="W6" s="19">
         <v>6308</v>
       </c>
-      <c r="X6" s="18"/>
-      <c r="Y6" s="18"/>
-      <c r="Z6" s="18"/>
-      <c r="AA6" s="18"/>
-      <c r="AB6" s="18"/>
-      <c r="AC6" s="18"/>
-      <c r="AD6" s="18"/>
-      <c r="AE6" s="18"/>
-      <c r="AF6" s="18" t="s">
+      <c r="X6" s="19"/>
+      <c r="Y6" s="19"/>
+      <c r="Z6" s="19"/>
+      <c r="AA6" s="19"/>
+      <c r="AB6" s="19"/>
+      <c r="AC6" s="19"/>
+      <c r="AD6" s="19"/>
+      <c r="AE6" s="19"/>
+      <c r="AF6" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="AG6" s="18"/>
-      <c r="AH6" s="18"/>
-      <c r="AI6" s="18"/>
-      <c r="AJ6" s="18"/>
-      <c r="AK6" s="18"/>
-      <c r="AL6" s="18"/>
-      <c r="AM6" s="18"/>
-      <c r="AN6" s="18"/>
+      <c r="AG6" s="19"/>
+      <c r="AH6" s="19"/>
+      <c r="AI6" s="19"/>
+      <c r="AJ6" s="19"/>
+      <c r="AK6" s="19"/>
+      <c r="AL6" s="19"/>
+      <c r="AM6" s="19"/>
+      <c r="AN6" s="19"/>
     </row>
     <row r="7" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="C7" s="17"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="17"/>
-      <c r="G7" s="17"/>
-      <c r="H7" s="17"/>
-      <c r="I7" s="17"/>
-      <c r="J7" s="17"/>
-      <c r="K7" s="17"/>
-      <c r="L7" s="17"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="17"/>
-      <c r="O7" s="17"/>
-      <c r="P7" s="17"/>
-      <c r="Q7" s="17"/>
-      <c r="R7" s="17"/>
-      <c r="S7" s="17"/>
-      <c r="T7" s="17"/>
-      <c r="U7" s="17"/>
-      <c r="V7" s="17"/>
-      <c r="W7" s="17">
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="18"/>
+      <c r="J7" s="18"/>
+      <c r="K7" s="18"/>
+      <c r="L7" s="18"/>
+      <c r="M7" s="18"/>
+      <c r="N7" s="18"/>
+      <c r="O7" s="18"/>
+      <c r="P7" s="18"/>
+      <c r="Q7" s="18"/>
+      <c r="R7" s="18"/>
+      <c r="S7" s="18"/>
+      <c r="T7" s="18"/>
+      <c r="U7" s="18"/>
+      <c r="V7" s="18"/>
+      <c r="W7" s="18">
         <v>7976</v>
       </c>
-      <c r="X7" s="17"/>
-      <c r="Y7" s="17"/>
-      <c r="Z7" s="17"/>
-      <c r="AA7" s="17"/>
-      <c r="AB7" s="17"/>
-      <c r="AC7" s="17"/>
-      <c r="AD7" s="17"/>
-      <c r="AE7" s="17"/>
-      <c r="AF7" s="17" t="s">
+      <c r="X7" s="18"/>
+      <c r="Y7" s="18"/>
+      <c r="Z7" s="18"/>
+      <c r="AA7" s="18"/>
+      <c r="AB7" s="18"/>
+      <c r="AC7" s="18"/>
+      <c r="AD7" s="18"/>
+      <c r="AE7" s="18"/>
+      <c r="AF7" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="AG7" s="17"/>
-      <c r="AH7" s="17"/>
-      <c r="AI7" s="17"/>
-      <c r="AJ7" s="17"/>
-      <c r="AK7" s="17"/>
-      <c r="AL7" s="17"/>
-      <c r="AM7" s="17"/>
-      <c r="AN7" s="17"/>
+      <c r="AG7" s="18"/>
+      <c r="AH7" s="18"/>
+      <c r="AI7" s="18"/>
+      <c r="AJ7" s="18"/>
+      <c r="AK7" s="18"/>
+      <c r="AL7" s="18"/>
+      <c r="AM7" s="18"/>
+      <c r="AN7" s="18"/>
     </row>
     <row r="8" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
-      <c r="O8" s="18"/>
-      <c r="P8" s="18"/>
-      <c r="Q8" s="18"/>
-      <c r="R8" s="18"/>
-      <c r="S8" s="18"/>
-      <c r="T8" s="18"/>
-      <c r="U8" s="18"/>
-      <c r="V8" s="18"/>
-      <c r="W8" s="18">
+      <c r="C8" s="19"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
+      <c r="F8" s="19"/>
+      <c r="G8" s="19"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="19"/>
+      <c r="L8" s="19"/>
+      <c r="M8" s="19"/>
+      <c r="N8" s="19"/>
+      <c r="O8" s="19"/>
+      <c r="P8" s="19"/>
+      <c r="Q8" s="19"/>
+      <c r="R8" s="19"/>
+      <c r="S8" s="19"/>
+      <c r="T8" s="19"/>
+      <c r="U8" s="19"/>
+      <c r="V8" s="19"/>
+      <c r="W8" s="19">
         <v>7572</v>
       </c>
-      <c r="X8" s="18"/>
-      <c r="Y8" s="18"/>
-      <c r="Z8" s="18"/>
-      <c r="AA8" s="18"/>
-      <c r="AB8" s="18"/>
-      <c r="AC8" s="18"/>
-      <c r="AD8" s="18"/>
-      <c r="AE8" s="18"/>
-      <c r="AF8" s="18" t="s">
+      <c r="X8" s="19"/>
+      <c r="Y8" s="19"/>
+      <c r="Z8" s="19"/>
+      <c r="AA8" s="19"/>
+      <c r="AB8" s="19"/>
+      <c r="AC8" s="19"/>
+      <c r="AD8" s="19"/>
+      <c r="AE8" s="19"/>
+      <c r="AF8" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="AG8" s="18"/>
-      <c r="AH8" s="18"/>
-      <c r="AI8" s="18"/>
-      <c r="AJ8" s="18"/>
-      <c r="AK8" s="18"/>
-      <c r="AL8" s="18"/>
-      <c r="AM8" s="18"/>
-      <c r="AN8" s="18"/>
+      <c r="AG8" s="19"/>
+      <c r="AH8" s="19"/>
+      <c r="AI8" s="19"/>
+      <c r="AJ8" s="19"/>
+      <c r="AK8" s="19"/>
+      <c r="AL8" s="19"/>
+      <c r="AM8" s="19"/>
+      <c r="AN8" s="19"/>
     </row>
     <row r="9" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B9" s="17" t="s">
+      <c r="B9" s="18" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="17"/>
-      <c r="D9" s="17"/>
-      <c r="E9" s="17"/>
-      <c r="F9" s="17"/>
-      <c r="G9" s="17"/>
-      <c r="H9" s="17"/>
-      <c r="I9" s="17"/>
-      <c r="J9" s="17"/>
-      <c r="K9" s="17"/>
-      <c r="L9" s="17"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="17"/>
-      <c r="O9" s="17"/>
-      <c r="P9" s="17"/>
-      <c r="Q9" s="17"/>
-      <c r="R9" s="17"/>
-      <c r="S9" s="17"/>
-      <c r="T9" s="17"/>
-      <c r="U9" s="17"/>
-      <c r="V9" s="17"/>
-      <c r="W9" s="17">
+      <c r="C9" s="18"/>
+      <c r="D9" s="18"/>
+      <c r="E9" s="18"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="18"/>
+      <c r="J9" s="18"/>
+      <c r="K9" s="18"/>
+      <c r="L9" s="18"/>
+      <c r="M9" s="18"/>
+      <c r="N9" s="18"/>
+      <c r="O9" s="18"/>
+      <c r="P9" s="18"/>
+      <c r="Q9" s="18"/>
+      <c r="R9" s="18"/>
+      <c r="S9" s="18"/>
+      <c r="T9" s="18"/>
+      <c r="U9" s="18"/>
+      <c r="V9" s="18"/>
+      <c r="W9" s="18">
         <v>8352</v>
       </c>
-      <c r="X9" s="17"/>
-      <c r="Y9" s="17"/>
-      <c r="Z9" s="17"/>
-      <c r="AA9" s="17"/>
-      <c r="AB9" s="17"/>
-      <c r="AC9" s="17"/>
-      <c r="AD9" s="17"/>
-      <c r="AE9" s="17"/>
-      <c r="AF9" s="17" t="s">
+      <c r="X9" s="18"/>
+      <c r="Y9" s="18"/>
+      <c r="Z9" s="18"/>
+      <c r="AA9" s="18"/>
+      <c r="AB9" s="18"/>
+      <c r="AC9" s="18"/>
+      <c r="AD9" s="18"/>
+      <c r="AE9" s="18"/>
+      <c r="AF9" s="18" t="s">
         <v>32</v>
       </c>
-      <c r="AG9" s="17"/>
-      <c r="AH9" s="17"/>
-      <c r="AI9" s="17"/>
-      <c r="AJ9" s="17"/>
-      <c r="AK9" s="17"/>
-      <c r="AL9" s="17"/>
-      <c r="AM9" s="17"/>
-      <c r="AN9" s="17"/>
+      <c r="AG9" s="18"/>
+      <c r="AH9" s="18"/>
+      <c r="AI9" s="18"/>
+      <c r="AJ9" s="18"/>
+      <c r="AK9" s="18"/>
+      <c r="AL9" s="18"/>
+      <c r="AM9" s="18"/>
+      <c r="AN9" s="18"/>
     </row>
     <row r="10" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B10" s="18" t="s">
+      <c r="B10" s="19" t="s">
         <v>33</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="18"/>
-      <c r="L10" s="18"/>
-      <c r="M10" s="18"/>
-      <c r="N10" s="18"/>
-      <c r="O10" s="18"/>
-      <c r="P10" s="18"/>
-      <c r="Q10" s="18"/>
-      <c r="R10" s="18"/>
-      <c r="S10" s="18"/>
-      <c r="T10" s="18"/>
-      <c r="U10" s="18"/>
-      <c r="V10" s="18"/>
-      <c r="W10" s="18">
+      <c r="C10" s="19"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
+      <c r="F10" s="19"/>
+      <c r="G10" s="19"/>
+      <c r="H10" s="19"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="19"/>
+      <c r="K10" s="19"/>
+      <c r="L10" s="19"/>
+      <c r="M10" s="19"/>
+      <c r="N10" s="19"/>
+      <c r="O10" s="19"/>
+      <c r="P10" s="19"/>
+      <c r="Q10" s="19"/>
+      <c r="R10" s="19"/>
+      <c r="S10" s="19"/>
+      <c r="T10" s="19"/>
+      <c r="U10" s="19"/>
+      <c r="V10" s="19"/>
+      <c r="W10" s="19">
         <v>15268</v>
       </c>
-      <c r="X10" s="18"/>
-      <c r="Y10" s="18"/>
-      <c r="Z10" s="18"/>
-      <c r="AA10" s="18"/>
-      <c r="AB10" s="18"/>
-      <c r="AC10" s="18"/>
-      <c r="AD10" s="18"/>
-      <c r="AE10" s="18"/>
-      <c r="AF10" s="18" t="s">
+      <c r="X10" s="19"/>
+      <c r="Y10" s="19"/>
+      <c r="Z10" s="19"/>
+      <c r="AA10" s="19"/>
+      <c r="AB10" s="19"/>
+      <c r="AC10" s="19"/>
+      <c r="AD10" s="19"/>
+      <c r="AE10" s="19"/>
+      <c r="AF10" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="AG10" s="18"/>
-      <c r="AH10" s="18"/>
-      <c r="AI10" s="18"/>
-      <c r="AJ10" s="18"/>
-      <c r="AK10" s="18"/>
-      <c r="AL10" s="18"/>
-      <c r="AM10" s="18"/>
-      <c r="AN10" s="18"/>
+      <c r="AG10" s="19"/>
+      <c r="AH10" s="19"/>
+      <c r="AI10" s="19"/>
+      <c r="AJ10" s="19"/>
+      <c r="AK10" s="19"/>
+      <c r="AL10" s="19"/>
+      <c r="AM10" s="19"/>
+      <c r="AN10" s="19"/>
     </row>
     <row r="11" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="17"/>
-      <c r="G11" s="17"/>
-      <c r="H11" s="17"/>
-      <c r="I11" s="17"/>
-      <c r="J11" s="17"/>
-      <c r="K11" s="17"/>
-      <c r="L11" s="17"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="17"/>
-      <c r="O11" s="17"/>
-      <c r="P11" s="17"/>
-      <c r="Q11" s="17"/>
-      <c r="R11" s="17"/>
-      <c r="S11" s="17"/>
-      <c r="T11" s="17"/>
-      <c r="U11" s="17"/>
-      <c r="V11" s="17"/>
-      <c r="W11" s="17">
+      <c r="C11" s="18"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="18"/>
+      <c r="J11" s="18"/>
+      <c r="K11" s="18"/>
+      <c r="L11" s="18"/>
+      <c r="M11" s="18"/>
+      <c r="N11" s="18"/>
+      <c r="O11" s="18"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="18"/>
+      <c r="R11" s="18"/>
+      <c r="S11" s="18"/>
+      <c r="T11" s="18"/>
+      <c r="U11" s="18"/>
+      <c r="V11" s="18"/>
+      <c r="W11" s="18">
         <v>5032</v>
       </c>
-      <c r="X11" s="17"/>
-      <c r="Y11" s="17"/>
-      <c r="Z11" s="17"/>
-      <c r="AA11" s="17"/>
-      <c r="AB11" s="17"/>
-      <c r="AC11" s="17"/>
-      <c r="AD11" s="17"/>
-      <c r="AE11" s="17"/>
-      <c r="AF11" s="17" t="s">
+      <c r="X11" s="18"/>
+      <c r="Y11" s="18"/>
+      <c r="Z11" s="18"/>
+      <c r="AA11" s="18"/>
+      <c r="AB11" s="18"/>
+      <c r="AC11" s="18"/>
+      <c r="AD11" s="18"/>
+      <c r="AE11" s="18"/>
+      <c r="AF11" s="18" t="s">
         <v>36</v>
       </c>
-      <c r="AG11" s="17"/>
-      <c r="AH11" s="17"/>
-      <c r="AI11" s="17"/>
-      <c r="AJ11" s="17"/>
-      <c r="AK11" s="17"/>
-      <c r="AL11" s="17"/>
-      <c r="AM11" s="17"/>
-      <c r="AN11" s="17"/>
+      <c r="AG11" s="18"/>
+      <c r="AH11" s="18"/>
+      <c r="AI11" s="18"/>
+      <c r="AJ11" s="18"/>
+      <c r="AK11" s="18"/>
+      <c r="AL11" s="18"/>
+      <c r="AM11" s="18"/>
+      <c r="AN11" s="18"/>
     </row>
     <row r="12" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B12" s="18" t="s">
+      <c r="B12" s="19" t="s">
         <v>37</v>
       </c>
-      <c r="C12" s="18"/>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="18"/>
-      <c r="I12" s="18"/>
-      <c r="J12" s="18"/>
-      <c r="K12" s="18"/>
-      <c r="L12" s="18"/>
-      <c r="M12" s="18"/>
-      <c r="N12" s="18"/>
-      <c r="O12" s="18"/>
-      <c r="P12" s="18"/>
-      <c r="Q12" s="18"/>
-      <c r="R12" s="18"/>
-      <c r="S12" s="18"/>
-      <c r="T12" s="18"/>
-      <c r="U12" s="18"/>
-      <c r="V12" s="18"/>
-      <c r="W12" s="18">
+      <c r="C12" s="19"/>
+      <c r="D12" s="19"/>
+      <c r="E12" s="19"/>
+      <c r="F12" s="19"/>
+      <c r="G12" s="19"/>
+      <c r="H12" s="19"/>
+      <c r="I12" s="19"/>
+      <c r="J12" s="19"/>
+      <c r="K12" s="19"/>
+      <c r="L12" s="19"/>
+      <c r="M12" s="19"/>
+      <c r="N12" s="19"/>
+      <c r="O12" s="19"/>
+      <c r="P12" s="19"/>
+      <c r="Q12" s="19"/>
+      <c r="R12" s="19"/>
+      <c r="S12" s="19"/>
+      <c r="T12" s="19"/>
+      <c r="U12" s="19"/>
+      <c r="V12" s="19"/>
+      <c r="W12" s="19">
         <v>17596</v>
       </c>
-      <c r="X12" s="18"/>
-      <c r="Y12" s="18"/>
-      <c r="Z12" s="18"/>
-      <c r="AA12" s="18"/>
-      <c r="AB12" s="18"/>
-      <c r="AC12" s="18"/>
-      <c r="AD12" s="18"/>
-      <c r="AE12" s="18"/>
-      <c r="AF12" s="18" t="s">
+      <c r="X12" s="19"/>
+      <c r="Y12" s="19"/>
+      <c r="Z12" s="19"/>
+      <c r="AA12" s="19"/>
+      <c r="AB12" s="19"/>
+      <c r="AC12" s="19"/>
+      <c r="AD12" s="19"/>
+      <c r="AE12" s="19"/>
+      <c r="AF12" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AG12" s="18"/>
-      <c r="AH12" s="18"/>
-      <c r="AI12" s="18"/>
-      <c r="AJ12" s="18"/>
-      <c r="AK12" s="18"/>
-      <c r="AL12" s="18"/>
-      <c r="AM12" s="18"/>
-      <c r="AN12" s="18"/>
+      <c r="AG12" s="19"/>
+      <c r="AH12" s="19"/>
+      <c r="AI12" s="19"/>
+      <c r="AJ12" s="19"/>
+      <c r="AK12" s="19"/>
+      <c r="AL12" s="19"/>
+      <c r="AM12" s="19"/>
+      <c r="AN12" s="19"/>
     </row>
     <row r="13" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B13" s="17" t="s">
+      <c r="B13" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="C13" s="17"/>
-      <c r="D13" s="17"/>
-      <c r="E13" s="17"/>
-      <c r="F13" s="17"/>
-      <c r="G13" s="17"/>
-      <c r="H13" s="17"/>
-      <c r="I13" s="17"/>
-      <c r="J13" s="17"/>
-      <c r="K13" s="17"/>
-      <c r="L13" s="17"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="17"/>
-      <c r="O13" s="17"/>
-      <c r="P13" s="17"/>
-      <c r="Q13" s="17"/>
-      <c r="R13" s="17"/>
-      <c r="S13" s="17"/>
-      <c r="T13" s="17"/>
-      <c r="U13" s="17"/>
-      <c r="V13" s="17"/>
-      <c r="W13" s="17">
+      <c r="C13" s="18"/>
+      <c r="D13" s="18"/>
+      <c r="E13" s="18"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="18"/>
+      <c r="J13" s="18"/>
+      <c r="K13" s="18"/>
+      <c r="L13" s="18"/>
+      <c r="M13" s="18"/>
+      <c r="N13" s="18"/>
+      <c r="O13" s="18"/>
+      <c r="P13" s="18"/>
+      <c r="Q13" s="18"/>
+      <c r="R13" s="18"/>
+      <c r="S13" s="18"/>
+      <c r="T13" s="18"/>
+      <c r="U13" s="18"/>
+      <c r="V13" s="18"/>
+      <c r="W13" s="18">
         <v>18748</v>
       </c>
-      <c r="X13" s="17"/>
-      <c r="Y13" s="17"/>
-      <c r="Z13" s="17"/>
-      <c r="AA13" s="17"/>
-      <c r="AB13" s="17"/>
-      <c r="AC13" s="17"/>
-      <c r="AD13" s="17"/>
-      <c r="AE13" s="17"/>
-      <c r="AF13" s="17" t="s">
+      <c r="X13" s="18"/>
+      <c r="Y13" s="18"/>
+      <c r="Z13" s="18"/>
+      <c r="AA13" s="18"/>
+      <c r="AB13" s="18"/>
+      <c r="AC13" s="18"/>
+      <c r="AD13" s="18"/>
+      <c r="AE13" s="18"/>
+      <c r="AF13" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="AG13" s="17"/>
-      <c r="AH13" s="17"/>
-      <c r="AI13" s="17"/>
-      <c r="AJ13" s="17"/>
-      <c r="AK13" s="17"/>
-      <c r="AL13" s="17"/>
-      <c r="AM13" s="17"/>
-      <c r="AN13" s="17"/>
+      <c r="AG13" s="18"/>
+      <c r="AH13" s="18"/>
+      <c r="AI13" s="18"/>
+      <c r="AJ13" s="18"/>
+      <c r="AK13" s="18"/>
+      <c r="AL13" s="18"/>
+      <c r="AM13" s="18"/>
+      <c r="AN13" s="18"/>
     </row>
     <row r="14" spans="1:40" x14ac:dyDescent="0.25">
-      <c r="B14" s="18" t="s">
+      <c r="B14" s="19" t="s">
         <v>41</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="18"/>
-      <c r="L14" s="18"/>
-      <c r="M14" s="18"/>
-      <c r="N14" s="18"/>
-      <c r="O14" s="18"/>
-      <c r="P14" s="18"/>
-      <c r="Q14" s="18"/>
-      <c r="R14" s="18"/>
-      <c r="S14" s="18"/>
-      <c r="T14" s="18"/>
-      <c r="U14" s="18"/>
-      <c r="V14" s="18"/>
-      <c r="W14" s="18">
+      <c r="C14" s="19"/>
+      <c r="D14" s="19"/>
+      <c r="E14" s="19"/>
+      <c r="F14" s="19"/>
+      <c r="G14" s="19"/>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
+      <c r="K14" s="19"/>
+      <c r="L14" s="19"/>
+      <c r="M14" s="19"/>
+      <c r="N14" s="19"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
+      <c r="Q14" s="19"/>
+      <c r="R14" s="19"/>
+      <c r="S14" s="19"/>
+      <c r="T14" s="19"/>
+      <c r="U14" s="19"/>
+      <c r="V14" s="19"/>
+      <c r="W14" s="19">
         <v>19292</v>
       </c>
-      <c r="X14" s="18"/>
-      <c r="Y14" s="18"/>
-      <c r="Z14" s="18"/>
-      <c r="AA14" s="18"/>
-      <c r="AB14" s="18"/>
-      <c r="AC14" s="18"/>
-      <c r="AD14" s="18"/>
-      <c r="AE14" s="18"/>
-      <c r="AF14" s="18" t="s">
+      <c r="X14" s="19"/>
+      <c r="Y14" s="19"/>
+      <c r="Z14" s="19"/>
+      <c r="AA14" s="19"/>
+      <c r="AB14" s="19"/>
+      <c r="AC14" s="19"/>
+      <c r="AD14" s="19"/>
+      <c r="AE14" s="19"/>
+      <c r="AF14" s="19" t="s">
         <v>42</v>
       </c>
-      <c r="AG14" s="18"/>
-      <c r="AH14" s="18"/>
-      <c r="AI14" s="18"/>
-      <c r="AJ14" s="18"/>
-      <c r="AK14" s="18"/>
-      <c r="AL14" s="18"/>
-      <c r="AM14" s="18"/>
-      <c r="AN14" s="18"/>
+      <c r="AG14" s="19"/>
+      <c r="AH14" s="19"/>
+      <c r="AI14" s="19"/>
+      <c r="AJ14" s="19"/>
+      <c r="AK14" s="19"/>
+      <c r="AL14" s="19"/>
+      <c r="AM14" s="19"/>
+      <c r="AN14" s="19"/>
     </row>
     <row r="16" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
@@ -1200,182 +1200,182 @@
       <c r="A18" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="19" t="s">
+      <c r="B18" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="19"/>
-      <c r="D18" s="19"/>
-      <c r="E18" s="19"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="19"/>
-      <c r="J18" s="19"/>
-      <c r="K18" s="19"/>
-      <c r="L18" s="19"/>
-      <c r="M18" s="19"/>
-      <c r="N18" s="19"/>
-      <c r="O18" s="19"/>
-      <c r="P18" s="19"/>
-      <c r="Q18" s="19"/>
-      <c r="R18" s="19"/>
-      <c r="S18" s="19"/>
-      <c r="T18" s="19"/>
-      <c r="U18" s="19"/>
-      <c r="V18" s="19"/>
-      <c r="W18" s="19"/>
-      <c r="X18" s="19"/>
-      <c r="Y18" s="19"/>
-      <c r="Z18" s="19"/>
-      <c r="AA18" s="19"/>
-      <c r="AB18" s="19"/>
-      <c r="AC18" s="19"/>
-      <c r="AD18" s="19"/>
-      <c r="AE18" s="19"/>
-      <c r="AF18" s="19"/>
-      <c r="AG18" s="19"/>
-      <c r="AH18" s="19"/>
-      <c r="AI18" s="19"/>
-      <c r="AJ18" s="19"/>
-      <c r="AK18" s="19"/>
-      <c r="AL18" s="19"/>
-      <c r="AM18" s="19"/>
-      <c r="AN18" s="19"/>
-      <c r="AO18" s="19"/>
-      <c r="AP18" s="19"/>
-      <c r="AQ18" s="19"/>
-      <c r="AR18" s="19"/>
-      <c r="AS18" s="19"/>
-      <c r="AT18" s="19"/>
-      <c r="AU18" s="19"/>
-      <c r="AV18" s="19"/>
-      <c r="AW18" s="19"/>
-      <c r="AX18" s="19"/>
-      <c r="AY18" s="19"/>
-      <c r="AZ18" s="19"/>
-      <c r="BA18" s="19"/>
-      <c r="BB18" s="19"/>
-      <c r="BC18" s="19"/>
-      <c r="BD18" s="19"/>
-      <c r="BE18" s="19"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
+      <c r="G18" s="17"/>
+      <c r="H18" s="17"/>
+      <c r="I18" s="17"/>
+      <c r="J18" s="17"/>
+      <c r="K18" s="17"/>
+      <c r="L18" s="17"/>
+      <c r="M18" s="17"/>
+      <c r="N18" s="17"/>
+      <c r="O18" s="17"/>
+      <c r="P18" s="17"/>
+      <c r="Q18" s="17"/>
+      <c r="R18" s="17"/>
+      <c r="S18" s="17"/>
+      <c r="T18" s="17"/>
+      <c r="U18" s="17"/>
+      <c r="V18" s="17"/>
+      <c r="W18" s="17"/>
+      <c r="X18" s="17"/>
+      <c r="Y18" s="17"/>
+      <c r="Z18" s="17"/>
+      <c r="AA18" s="17"/>
+      <c r="AB18" s="17"/>
+      <c r="AC18" s="17"/>
+      <c r="AD18" s="17"/>
+      <c r="AE18" s="17"/>
+      <c r="AF18" s="17"/>
+      <c r="AG18" s="17"/>
+      <c r="AH18" s="17"/>
+      <c r="AI18" s="17"/>
+      <c r="AJ18" s="17"/>
+      <c r="AK18" s="17"/>
+      <c r="AL18" s="17"/>
+      <c r="AM18" s="17"/>
+      <c r="AN18" s="17"/>
+      <c r="AO18" s="17"/>
+      <c r="AP18" s="17"/>
+      <c r="AQ18" s="17"/>
+      <c r="AR18" s="17"/>
+      <c r="AS18" s="17"/>
+      <c r="AT18" s="17"/>
+      <c r="AU18" s="17"/>
+      <c r="AV18" s="17"/>
+      <c r="AW18" s="17"/>
+      <c r="AX18" s="17"/>
+      <c r="AY18" s="17"/>
+      <c r="AZ18" s="17"/>
+      <c r="BA18" s="17"/>
+      <c r="BB18" s="17"/>
+      <c r="BC18" s="17"/>
+      <c r="BD18" s="17"/>
+      <c r="BE18" s="17"/>
     </row>
     <row r="19" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
-      <c r="B19" s="19"/>
-      <c r="C19" s="19"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="19"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="19"/>
-      <c r="K19" s="19"/>
-      <c r="L19" s="19"/>
-      <c r="M19" s="19"/>
-      <c r="N19" s="19"/>
-      <c r="O19" s="19"/>
-      <c r="P19" s="19"/>
-      <c r="Q19" s="19"/>
-      <c r="R19" s="19"/>
-      <c r="S19" s="19"/>
-      <c r="T19" s="19"/>
-      <c r="U19" s="19"/>
-      <c r="V19" s="19"/>
-      <c r="W19" s="19"/>
-      <c r="X19" s="19"/>
-      <c r="Y19" s="19"/>
-      <c r="Z19" s="19"/>
-      <c r="AA19" s="19"/>
-      <c r="AB19" s="19"/>
-      <c r="AC19" s="19"/>
-      <c r="AD19" s="19"/>
-      <c r="AE19" s="19"/>
-      <c r="AF19" s="19"/>
-      <c r="AG19" s="19"/>
-      <c r="AH19" s="19"/>
-      <c r="AI19" s="19"/>
-      <c r="AJ19" s="19"/>
-      <c r="AK19" s="19"/>
-      <c r="AL19" s="19"/>
-      <c r="AM19" s="19"/>
-      <c r="AN19" s="19"/>
-      <c r="AO19" s="19"/>
-      <c r="AP19" s="19"/>
-      <c r="AQ19" s="19"/>
-      <c r="AR19" s="19"/>
-      <c r="AS19" s="19"/>
-      <c r="AT19" s="19"/>
-      <c r="AU19" s="19"/>
-      <c r="AV19" s="19"/>
-      <c r="AW19" s="19"/>
-      <c r="AX19" s="19"/>
-      <c r="AY19" s="19"/>
-      <c r="AZ19" s="19"/>
-      <c r="BA19" s="19"/>
-      <c r="BB19" s="19"/>
-      <c r="BC19" s="19"/>
-      <c r="BD19" s="19"/>
-      <c r="BE19" s="19"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
+      <c r="G19" s="17"/>
+      <c r="H19" s="17"/>
+      <c r="I19" s="17"/>
+      <c r="J19" s="17"/>
+      <c r="K19" s="17"/>
+      <c r="L19" s="17"/>
+      <c r="M19" s="17"/>
+      <c r="N19" s="17"/>
+      <c r="O19" s="17"/>
+      <c r="P19" s="17"/>
+      <c r="Q19" s="17"/>
+      <c r="R19" s="17"/>
+      <c r="S19" s="17"/>
+      <c r="T19" s="17"/>
+      <c r="U19" s="17"/>
+      <c r="V19" s="17"/>
+      <c r="W19" s="17"/>
+      <c r="X19" s="17"/>
+      <c r="Y19" s="17"/>
+      <c r="Z19" s="17"/>
+      <c r="AA19" s="17"/>
+      <c r="AB19" s="17"/>
+      <c r="AC19" s="17"/>
+      <c r="AD19" s="17"/>
+      <c r="AE19" s="17"/>
+      <c r="AF19" s="17"/>
+      <c r="AG19" s="17"/>
+      <c r="AH19" s="17"/>
+      <c r="AI19" s="17"/>
+      <c r="AJ19" s="17"/>
+      <c r="AK19" s="17"/>
+      <c r="AL19" s="17"/>
+      <c r="AM19" s="17"/>
+      <c r="AN19" s="17"/>
+      <c r="AO19" s="17"/>
+      <c r="AP19" s="17"/>
+      <c r="AQ19" s="17"/>
+      <c r="AR19" s="17"/>
+      <c r="AS19" s="17"/>
+      <c r="AT19" s="17"/>
+      <c r="AU19" s="17"/>
+      <c r="AV19" s="17"/>
+      <c r="AW19" s="17"/>
+      <c r="AX19" s="17"/>
+      <c r="AY19" s="17"/>
+      <c r="AZ19" s="17"/>
+      <c r="BA19" s="17"/>
+      <c r="BB19" s="17"/>
+      <c r="BC19" s="17"/>
+      <c r="BD19" s="17"/>
+      <c r="BE19" s="17"/>
     </row>
     <row r="20" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
-      <c r="B20" s="19"/>
-      <c r="C20" s="19"/>
-      <c r="D20" s="19"/>
-      <c r="E20" s="19"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="19"/>
-      <c r="J20" s="19"/>
-      <c r="K20" s="19"/>
-      <c r="L20" s="19"/>
-      <c r="M20" s="19"/>
-      <c r="N20" s="19"/>
-      <c r="O20" s="19"/>
-      <c r="P20" s="19"/>
-      <c r="Q20" s="19"/>
-      <c r="R20" s="19"/>
-      <c r="S20" s="19"/>
-      <c r="T20" s="19"/>
-      <c r="U20" s="19"/>
-      <c r="V20" s="19"/>
-      <c r="W20" s="19"/>
-      <c r="X20" s="19"/>
-      <c r="Y20" s="19"/>
-      <c r="Z20" s="19"/>
-      <c r="AA20" s="19"/>
-      <c r="AB20" s="19"/>
-      <c r="AC20" s="19"/>
-      <c r="AD20" s="19"/>
-      <c r="AE20" s="19"/>
-      <c r="AF20" s="19"/>
-      <c r="AG20" s="19"/>
-      <c r="AH20" s="19"/>
-      <c r="AI20" s="19"/>
-      <c r="AJ20" s="19"/>
-      <c r="AK20" s="19"/>
-      <c r="AL20" s="19"/>
-      <c r="AM20" s="19"/>
-      <c r="AN20" s="19"/>
-      <c r="AO20" s="19"/>
-      <c r="AP20" s="19"/>
-      <c r="AQ20" s="19"/>
-      <c r="AR20" s="19"/>
-      <c r="AS20" s="19"/>
-      <c r="AT20" s="19"/>
-      <c r="AU20" s="19"/>
-      <c r="AV20" s="19"/>
-      <c r="AW20" s="19"/>
-      <c r="AX20" s="19"/>
-      <c r="AY20" s="19"/>
-      <c r="AZ20" s="19"/>
-      <c r="BA20" s="19"/>
-      <c r="BB20" s="19"/>
-      <c r="BC20" s="19"/>
-      <c r="BD20" s="19"/>
-      <c r="BE20" s="19"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
+      <c r="G20" s="17"/>
+      <c r="H20" s="17"/>
+      <c r="I20" s="17"/>
+      <c r="J20" s="17"/>
+      <c r="K20" s="17"/>
+      <c r="L20" s="17"/>
+      <c r="M20" s="17"/>
+      <c r="N20" s="17"/>
+      <c r="O20" s="17"/>
+      <c r="P20" s="17"/>
+      <c r="Q20" s="17"/>
+      <c r="R20" s="17"/>
+      <c r="S20" s="17"/>
+      <c r="T20" s="17"/>
+      <c r="U20" s="17"/>
+      <c r="V20" s="17"/>
+      <c r="W20" s="17"/>
+      <c r="X20" s="17"/>
+      <c r="Y20" s="17"/>
+      <c r="Z20" s="17"/>
+      <c r="AA20" s="17"/>
+      <c r="AB20" s="17"/>
+      <c r="AC20" s="17"/>
+      <c r="AD20" s="17"/>
+      <c r="AE20" s="17"/>
+      <c r="AF20" s="17"/>
+      <c r="AG20" s="17"/>
+      <c r="AH20" s="17"/>
+      <c r="AI20" s="17"/>
+      <c r="AJ20" s="17"/>
+      <c r="AK20" s="17"/>
+      <c r="AL20" s="17"/>
+      <c r="AM20" s="17"/>
+      <c r="AN20" s="17"/>
+      <c r="AO20" s="17"/>
+      <c r="AP20" s="17"/>
+      <c r="AQ20" s="17"/>
+      <c r="AR20" s="17"/>
+      <c r="AS20" s="17"/>
+      <c r="AT20" s="17"/>
+      <c r="AU20" s="17"/>
+      <c r="AV20" s="17"/>
+      <c r="AW20" s="17"/>
+      <c r="AX20" s="17"/>
+      <c r="AY20" s="17"/>
+      <c r="AZ20" s="17"/>
+      <c r="BA20" s="17"/>
+      <c r="BB20" s="17"/>
+      <c r="BC20" s="17"/>
+      <c r="BD20" s="17"/>
+      <c r="BE20" s="17"/>
     </row>
     <row r="22" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A22" s="7">
@@ -1389,182 +1389,182 @@
       <c r="A23" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="19" t="s">
+      <c r="B23" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C23" s="19"/>
-      <c r="D23" s="19"/>
-      <c r="E23" s="19"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="19"/>
-      <c r="J23" s="19"/>
-      <c r="K23" s="19"/>
-      <c r="L23" s="19"/>
-      <c r="M23" s="19"/>
-      <c r="N23" s="19"/>
-      <c r="O23" s="19"/>
-      <c r="P23" s="19"/>
-      <c r="Q23" s="19"/>
-      <c r="R23" s="19"/>
-      <c r="S23" s="19"/>
-      <c r="T23" s="19"/>
-      <c r="U23" s="19"/>
-      <c r="V23" s="19"/>
-      <c r="W23" s="19"/>
-      <c r="X23" s="19"/>
-      <c r="Y23" s="19"/>
-      <c r="Z23" s="19"/>
-      <c r="AA23" s="19"/>
-      <c r="AB23" s="19"/>
-      <c r="AC23" s="19"/>
-      <c r="AD23" s="19"/>
-      <c r="AE23" s="19"/>
-      <c r="AF23" s="19"/>
-      <c r="AG23" s="19"/>
-      <c r="AH23" s="19"/>
-      <c r="AI23" s="19"/>
-      <c r="AJ23" s="19"/>
-      <c r="AK23" s="19"/>
-      <c r="AL23" s="19"/>
-      <c r="AM23" s="19"/>
-      <c r="AN23" s="19"/>
-      <c r="AO23" s="19"/>
-      <c r="AP23" s="19"/>
-      <c r="AQ23" s="19"/>
-      <c r="AR23" s="19"/>
-      <c r="AS23" s="19"/>
-      <c r="AT23" s="19"/>
-      <c r="AU23" s="19"/>
-      <c r="AV23" s="19"/>
-      <c r="AW23" s="19"/>
-      <c r="AX23" s="19"/>
-      <c r="AY23" s="19"/>
-      <c r="AZ23" s="19"/>
-      <c r="BA23" s="19"/>
-      <c r="BB23" s="19"/>
-      <c r="BC23" s="19"/>
-      <c r="BD23" s="19"/>
-      <c r="BE23" s="19"/>
+      <c r="C23" s="17"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
+      <c r="G23" s="17"/>
+      <c r="H23" s="17"/>
+      <c r="I23" s="17"/>
+      <c r="J23" s="17"/>
+      <c r="K23" s="17"/>
+      <c r="L23" s="17"/>
+      <c r="M23" s="17"/>
+      <c r="N23" s="17"/>
+      <c r="O23" s="17"/>
+      <c r="P23" s="17"/>
+      <c r="Q23" s="17"/>
+      <c r="R23" s="17"/>
+      <c r="S23" s="17"/>
+      <c r="T23" s="17"/>
+      <c r="U23" s="17"/>
+      <c r="V23" s="17"/>
+      <c r="W23" s="17"/>
+      <c r="X23" s="17"/>
+      <c r="Y23" s="17"/>
+      <c r="Z23" s="17"/>
+      <c r="AA23" s="17"/>
+      <c r="AB23" s="17"/>
+      <c r="AC23" s="17"/>
+      <c r="AD23" s="17"/>
+      <c r="AE23" s="17"/>
+      <c r="AF23" s="17"/>
+      <c r="AG23" s="17"/>
+      <c r="AH23" s="17"/>
+      <c r="AI23" s="17"/>
+      <c r="AJ23" s="17"/>
+      <c r="AK23" s="17"/>
+      <c r="AL23" s="17"/>
+      <c r="AM23" s="17"/>
+      <c r="AN23" s="17"/>
+      <c r="AO23" s="17"/>
+      <c r="AP23" s="17"/>
+      <c r="AQ23" s="17"/>
+      <c r="AR23" s="17"/>
+      <c r="AS23" s="17"/>
+      <c r="AT23" s="17"/>
+      <c r="AU23" s="17"/>
+      <c r="AV23" s="17"/>
+      <c r="AW23" s="17"/>
+      <c r="AX23" s="17"/>
+      <c r="AY23" s="17"/>
+      <c r="AZ23" s="17"/>
+      <c r="BA23" s="17"/>
+      <c r="BB23" s="17"/>
+      <c r="BC23" s="17"/>
+      <c r="BD23" s="17"/>
+      <c r="BE23" s="17"/>
     </row>
     <row r="24" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="19"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="19"/>
-      <c r="J24" s="19"/>
-      <c r="K24" s="19"/>
-      <c r="L24" s="19"/>
-      <c r="M24" s="19"/>
-      <c r="N24" s="19"/>
-      <c r="O24" s="19"/>
-      <c r="P24" s="19"/>
-      <c r="Q24" s="19"/>
-      <c r="R24" s="19"/>
-      <c r="S24" s="19"/>
-      <c r="T24" s="19"/>
-      <c r="U24" s="19"/>
-      <c r="V24" s="19"/>
-      <c r="W24" s="19"/>
-      <c r="X24" s="19"/>
-      <c r="Y24" s="19"/>
-      <c r="Z24" s="19"/>
-      <c r="AA24" s="19"/>
-      <c r="AB24" s="19"/>
-      <c r="AC24" s="19"/>
-      <c r="AD24" s="19"/>
-      <c r="AE24" s="19"/>
-      <c r="AF24" s="19"/>
-      <c r="AG24" s="19"/>
-      <c r="AH24" s="19"/>
-      <c r="AI24" s="19"/>
-      <c r="AJ24" s="19"/>
-      <c r="AK24" s="19"/>
-      <c r="AL24" s="19"/>
-      <c r="AM24" s="19"/>
-      <c r="AN24" s="19"/>
-      <c r="AO24" s="19"/>
-      <c r="AP24" s="19"/>
-      <c r="AQ24" s="19"/>
-      <c r="AR24" s="19"/>
-      <c r="AS24" s="19"/>
-      <c r="AT24" s="19"/>
-      <c r="AU24" s="19"/>
-      <c r="AV24" s="19"/>
-      <c r="AW24" s="19"/>
-      <c r="AX24" s="19"/>
-      <c r="AY24" s="19"/>
-      <c r="AZ24" s="19"/>
-      <c r="BA24" s="19"/>
-      <c r="BB24" s="19"/>
-      <c r="BC24" s="19"/>
-      <c r="BD24" s="19"/>
-      <c r="BE24" s="19"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
+      <c r="G24" s="17"/>
+      <c r="H24" s="17"/>
+      <c r="I24" s="17"/>
+      <c r="J24" s="17"/>
+      <c r="K24" s="17"/>
+      <c r="L24" s="17"/>
+      <c r="M24" s="17"/>
+      <c r="N24" s="17"/>
+      <c r="O24" s="17"/>
+      <c r="P24" s="17"/>
+      <c r="Q24" s="17"/>
+      <c r="R24" s="17"/>
+      <c r="S24" s="17"/>
+      <c r="T24" s="17"/>
+      <c r="U24" s="17"/>
+      <c r="V24" s="17"/>
+      <c r="W24" s="17"/>
+      <c r="X24" s="17"/>
+      <c r="Y24" s="17"/>
+      <c r="Z24" s="17"/>
+      <c r="AA24" s="17"/>
+      <c r="AB24" s="17"/>
+      <c r="AC24" s="17"/>
+      <c r="AD24" s="17"/>
+      <c r="AE24" s="17"/>
+      <c r="AF24" s="17"/>
+      <c r="AG24" s="17"/>
+      <c r="AH24" s="17"/>
+      <c r="AI24" s="17"/>
+      <c r="AJ24" s="17"/>
+      <c r="AK24" s="17"/>
+      <c r="AL24" s="17"/>
+      <c r="AM24" s="17"/>
+      <c r="AN24" s="17"/>
+      <c r="AO24" s="17"/>
+      <c r="AP24" s="17"/>
+      <c r="AQ24" s="17"/>
+      <c r="AR24" s="17"/>
+      <c r="AS24" s="17"/>
+      <c r="AT24" s="17"/>
+      <c r="AU24" s="17"/>
+      <c r="AV24" s="17"/>
+      <c r="AW24" s="17"/>
+      <c r="AX24" s="17"/>
+      <c r="AY24" s="17"/>
+      <c r="AZ24" s="17"/>
+      <c r="BA24" s="17"/>
+      <c r="BB24" s="17"/>
+      <c r="BC24" s="17"/>
+      <c r="BD24" s="17"/>
+      <c r="BE24" s="17"/>
     </row>
     <row r="25" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
-      <c r="B25" s="19"/>
-      <c r="C25" s="19"/>
-      <c r="D25" s="19"/>
-      <c r="E25" s="19"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="19"/>
-      <c r="J25" s="19"/>
-      <c r="K25" s="19"/>
-      <c r="L25" s="19"/>
-      <c r="M25" s="19"/>
-      <c r="N25" s="19"/>
-      <c r="O25" s="19"/>
-      <c r="P25" s="19"/>
-      <c r="Q25" s="19"/>
-      <c r="R25" s="19"/>
-      <c r="S25" s="19"/>
-      <c r="T25" s="19"/>
-      <c r="U25" s="19"/>
-      <c r="V25" s="19"/>
-      <c r="W25" s="19"/>
-      <c r="X25" s="19"/>
-      <c r="Y25" s="19"/>
-      <c r="Z25" s="19"/>
-      <c r="AA25" s="19"/>
-      <c r="AB25" s="19"/>
-      <c r="AC25" s="19"/>
-      <c r="AD25" s="19"/>
-      <c r="AE25" s="19"/>
-      <c r="AF25" s="19"/>
-      <c r="AG25" s="19"/>
-      <c r="AH25" s="19"/>
-      <c r="AI25" s="19"/>
-      <c r="AJ25" s="19"/>
-      <c r="AK25" s="19"/>
-      <c r="AL25" s="19"/>
-      <c r="AM25" s="19"/>
-      <c r="AN25" s="19"/>
-      <c r="AO25" s="19"/>
-      <c r="AP25" s="19"/>
-      <c r="AQ25" s="19"/>
-      <c r="AR25" s="19"/>
-      <c r="AS25" s="19"/>
-      <c r="AT25" s="19"/>
-      <c r="AU25" s="19"/>
-      <c r="AV25" s="19"/>
-      <c r="AW25" s="19"/>
-      <c r="AX25" s="19"/>
-      <c r="AY25" s="19"/>
-      <c r="AZ25" s="19"/>
-      <c r="BA25" s="19"/>
-      <c r="BB25" s="19"/>
-      <c r="BC25" s="19"/>
-      <c r="BD25" s="19"/>
-      <c r="BE25" s="19"/>
+      <c r="B25" s="17"/>
+      <c r="C25" s="17"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
+      <c r="G25" s="17"/>
+      <c r="H25" s="17"/>
+      <c r="I25" s="17"/>
+      <c r="J25" s="17"/>
+      <c r="K25" s="17"/>
+      <c r="L25" s="17"/>
+      <c r="M25" s="17"/>
+      <c r="N25" s="17"/>
+      <c r="O25" s="17"/>
+      <c r="P25" s="17"/>
+      <c r="Q25" s="17"/>
+      <c r="R25" s="17"/>
+      <c r="S25" s="17"/>
+      <c r="T25" s="17"/>
+      <c r="U25" s="17"/>
+      <c r="V25" s="17"/>
+      <c r="W25" s="17"/>
+      <c r="X25" s="17"/>
+      <c r="Y25" s="17"/>
+      <c r="Z25" s="17"/>
+      <c r="AA25" s="17"/>
+      <c r="AB25" s="17"/>
+      <c r="AC25" s="17"/>
+      <c r="AD25" s="17"/>
+      <c r="AE25" s="17"/>
+      <c r="AF25" s="17"/>
+      <c r="AG25" s="17"/>
+      <c r="AH25" s="17"/>
+      <c r="AI25" s="17"/>
+      <c r="AJ25" s="17"/>
+      <c r="AK25" s="17"/>
+      <c r="AL25" s="17"/>
+      <c r="AM25" s="17"/>
+      <c r="AN25" s="17"/>
+      <c r="AO25" s="17"/>
+      <c r="AP25" s="17"/>
+      <c r="AQ25" s="17"/>
+      <c r="AR25" s="17"/>
+      <c r="AS25" s="17"/>
+      <c r="AT25" s="17"/>
+      <c r="AU25" s="17"/>
+      <c r="AV25" s="17"/>
+      <c r="AW25" s="17"/>
+      <c r="AX25" s="17"/>
+      <c r="AY25" s="17"/>
+      <c r="AZ25" s="17"/>
+      <c r="BA25" s="17"/>
+      <c r="BB25" s="17"/>
+      <c r="BC25" s="17"/>
+      <c r="BD25" s="17"/>
+      <c r="BE25" s="17"/>
     </row>
     <row r="27" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A27" s="7">
@@ -1578,180 +1578,180 @@
       <c r="A28" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B28" s="19" t="s">
+      <c r="B28" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="19"/>
-      <c r="D28" s="19"/>
-      <c r="E28" s="19"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="19"/>
-      <c r="J28" s="19"/>
-      <c r="K28" s="19"/>
-      <c r="L28" s="19"/>
-      <c r="M28" s="19"/>
-      <c r="N28" s="19"/>
-      <c r="O28" s="19"/>
-      <c r="P28" s="19"/>
-      <c r="Q28" s="19"/>
-      <c r="R28" s="19"/>
-      <c r="S28" s="19"/>
-      <c r="T28" s="19"/>
-      <c r="U28" s="19"/>
-      <c r="V28" s="19"/>
-      <c r="W28" s="19"/>
-      <c r="X28" s="19"/>
-      <c r="Y28" s="19"/>
-      <c r="Z28" s="19"/>
-      <c r="AA28" s="19"/>
-      <c r="AB28" s="19"/>
-      <c r="AC28" s="19"/>
-      <c r="AD28" s="19"/>
-      <c r="AE28" s="19"/>
-      <c r="AF28" s="19"/>
-      <c r="AG28" s="19"/>
-      <c r="AH28" s="19"/>
-      <c r="AI28" s="19"/>
-      <c r="AJ28" s="19"/>
-      <c r="AK28" s="19"/>
-      <c r="AL28" s="19"/>
-      <c r="AM28" s="19"/>
-      <c r="AN28" s="19"/>
-      <c r="AO28" s="19"/>
-      <c r="AP28" s="19"/>
-      <c r="AQ28" s="19"/>
-      <c r="AR28" s="19"/>
-      <c r="AS28" s="19"/>
-      <c r="AT28" s="19"/>
-      <c r="AU28" s="19"/>
-      <c r="AV28" s="19"/>
-      <c r="AW28" s="19"/>
-      <c r="AX28" s="19"/>
-      <c r="AY28" s="19"/>
-      <c r="AZ28" s="19"/>
-      <c r="BA28" s="19"/>
-      <c r="BB28" s="19"/>
-      <c r="BC28" s="19"/>
-      <c r="BD28" s="19"/>
-      <c r="BE28" s="19"/>
+      <c r="C28" s="17"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="17"/>
+      <c r="H28" s="17"/>
+      <c r="I28" s="17"/>
+      <c r="J28" s="17"/>
+      <c r="K28" s="17"/>
+      <c r="L28" s="17"/>
+      <c r="M28" s="17"/>
+      <c r="N28" s="17"/>
+      <c r="O28" s="17"/>
+      <c r="P28" s="17"/>
+      <c r="Q28" s="17"/>
+      <c r="R28" s="17"/>
+      <c r="S28" s="17"/>
+      <c r="T28" s="17"/>
+      <c r="U28" s="17"/>
+      <c r="V28" s="17"/>
+      <c r="W28" s="17"/>
+      <c r="X28" s="17"/>
+      <c r="Y28" s="17"/>
+      <c r="Z28" s="17"/>
+      <c r="AA28" s="17"/>
+      <c r="AB28" s="17"/>
+      <c r="AC28" s="17"/>
+      <c r="AD28" s="17"/>
+      <c r="AE28" s="17"/>
+      <c r="AF28" s="17"/>
+      <c r="AG28" s="17"/>
+      <c r="AH28" s="17"/>
+      <c r="AI28" s="17"/>
+      <c r="AJ28" s="17"/>
+      <c r="AK28" s="17"/>
+      <c r="AL28" s="17"/>
+      <c r="AM28" s="17"/>
+      <c r="AN28" s="17"/>
+      <c r="AO28" s="17"/>
+      <c r="AP28" s="17"/>
+      <c r="AQ28" s="17"/>
+      <c r="AR28" s="17"/>
+      <c r="AS28" s="17"/>
+      <c r="AT28" s="17"/>
+      <c r="AU28" s="17"/>
+      <c r="AV28" s="17"/>
+      <c r="AW28" s="17"/>
+      <c r="AX28" s="17"/>
+      <c r="AY28" s="17"/>
+      <c r="AZ28" s="17"/>
+      <c r="BA28" s="17"/>
+      <c r="BB28" s="17"/>
+      <c r="BC28" s="17"/>
+      <c r="BD28" s="17"/>
+      <c r="BE28" s="17"/>
     </row>
     <row r="29" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="B29" s="19"/>
-      <c r="C29" s="19"/>
-      <c r="D29" s="19"/>
-      <c r="E29" s="19"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="19"/>
-      <c r="J29" s="19"/>
-      <c r="K29" s="19"/>
-      <c r="L29" s="19"/>
-      <c r="M29" s="19"/>
-      <c r="N29" s="19"/>
-      <c r="O29" s="19"/>
-      <c r="P29" s="19"/>
-      <c r="Q29" s="19"/>
-      <c r="R29" s="19"/>
-      <c r="S29" s="19"/>
-      <c r="T29" s="19"/>
-      <c r="U29" s="19"/>
-      <c r="V29" s="19"/>
-      <c r="W29" s="19"/>
-      <c r="X29" s="19"/>
-      <c r="Y29" s="19"/>
-      <c r="Z29" s="19"/>
-      <c r="AA29" s="19"/>
-      <c r="AB29" s="19"/>
-      <c r="AC29" s="19"/>
-      <c r="AD29" s="19"/>
-      <c r="AE29" s="19"/>
-      <c r="AF29" s="19"/>
-      <c r="AG29" s="19"/>
-      <c r="AH29" s="19"/>
-      <c r="AI29" s="19"/>
-      <c r="AJ29" s="19"/>
-      <c r="AK29" s="19"/>
-      <c r="AL29" s="19"/>
-      <c r="AM29" s="19"/>
-      <c r="AN29" s="19"/>
-      <c r="AO29" s="19"/>
-      <c r="AP29" s="19"/>
-      <c r="AQ29" s="19"/>
-      <c r="AR29" s="19"/>
-      <c r="AS29" s="19"/>
-      <c r="AT29" s="19"/>
-      <c r="AU29" s="19"/>
-      <c r="AV29" s="19"/>
-      <c r="AW29" s="19"/>
-      <c r="AX29" s="19"/>
-      <c r="AY29" s="19"/>
-      <c r="AZ29" s="19"/>
-      <c r="BA29" s="19"/>
-      <c r="BB29" s="19"/>
-      <c r="BC29" s="19"/>
-      <c r="BD29" s="19"/>
-      <c r="BE29" s="19"/>
+      <c r="B29" s="17"/>
+      <c r="C29" s="17"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="17"/>
+      <c r="H29" s="17"/>
+      <c r="I29" s="17"/>
+      <c r="J29" s="17"/>
+      <c r="K29" s="17"/>
+      <c r="L29" s="17"/>
+      <c r="M29" s="17"/>
+      <c r="N29" s="17"/>
+      <c r="O29" s="17"/>
+      <c r="P29" s="17"/>
+      <c r="Q29" s="17"/>
+      <c r="R29" s="17"/>
+      <c r="S29" s="17"/>
+      <c r="T29" s="17"/>
+      <c r="U29" s="17"/>
+      <c r="V29" s="17"/>
+      <c r="W29" s="17"/>
+      <c r="X29" s="17"/>
+      <c r="Y29" s="17"/>
+      <c r="Z29" s="17"/>
+      <c r="AA29" s="17"/>
+      <c r="AB29" s="17"/>
+      <c r="AC29" s="17"/>
+      <c r="AD29" s="17"/>
+      <c r="AE29" s="17"/>
+      <c r="AF29" s="17"/>
+      <c r="AG29" s="17"/>
+      <c r="AH29" s="17"/>
+      <c r="AI29" s="17"/>
+      <c r="AJ29" s="17"/>
+      <c r="AK29" s="17"/>
+      <c r="AL29" s="17"/>
+      <c r="AM29" s="17"/>
+      <c r="AN29" s="17"/>
+      <c r="AO29" s="17"/>
+      <c r="AP29" s="17"/>
+      <c r="AQ29" s="17"/>
+      <c r="AR29" s="17"/>
+      <c r="AS29" s="17"/>
+      <c r="AT29" s="17"/>
+      <c r="AU29" s="17"/>
+      <c r="AV29" s="17"/>
+      <c r="AW29" s="17"/>
+      <c r="AX29" s="17"/>
+      <c r="AY29" s="17"/>
+      <c r="AZ29" s="17"/>
+      <c r="BA29" s="17"/>
+      <c r="BB29" s="17"/>
+      <c r="BC29" s="17"/>
+      <c r="BD29" s="17"/>
+      <c r="BE29" s="17"/>
     </row>
     <row r="30" spans="1:57" x14ac:dyDescent="0.25">
-      <c r="B30" s="19"/>
-      <c r="C30" s="19"/>
-      <c r="D30" s="19"/>
-      <c r="E30" s="19"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="19"/>
-      <c r="J30" s="19"/>
-      <c r="K30" s="19"/>
-      <c r="L30" s="19"/>
-      <c r="M30" s="19"/>
-      <c r="N30" s="19"/>
-      <c r="O30" s="19"/>
-      <c r="P30" s="19"/>
-      <c r="Q30" s="19"/>
-      <c r="R30" s="19"/>
-      <c r="S30" s="19"/>
-      <c r="T30" s="19"/>
-      <c r="U30" s="19"/>
-      <c r="V30" s="19"/>
-      <c r="W30" s="19"/>
-      <c r="X30" s="19"/>
-      <c r="Y30" s="19"/>
-      <c r="Z30" s="19"/>
-      <c r="AA30" s="19"/>
-      <c r="AB30" s="19"/>
-      <c r="AC30" s="19"/>
-      <c r="AD30" s="19"/>
-      <c r="AE30" s="19"/>
-      <c r="AF30" s="19"/>
-      <c r="AG30" s="19"/>
-      <c r="AH30" s="19"/>
-      <c r="AI30" s="19"/>
-      <c r="AJ30" s="19"/>
-      <c r="AK30" s="19"/>
-      <c r="AL30" s="19"/>
-      <c r="AM30" s="19"/>
-      <c r="AN30" s="19"/>
-      <c r="AO30" s="19"/>
-      <c r="AP30" s="19"/>
-      <c r="AQ30" s="19"/>
-      <c r="AR30" s="19"/>
-      <c r="AS30" s="19"/>
-      <c r="AT30" s="19"/>
-      <c r="AU30" s="19"/>
-      <c r="AV30" s="19"/>
-      <c r="AW30" s="19"/>
-      <c r="AX30" s="19"/>
-      <c r="AY30" s="19"/>
-      <c r="AZ30" s="19"/>
-      <c r="BA30" s="19"/>
-      <c r="BB30" s="19"/>
-      <c r="BC30" s="19"/>
-      <c r="BD30" s="19"/>
-      <c r="BE30" s="19"/>
+      <c r="B30" s="17"/>
+      <c r="C30" s="17"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="17"/>
+      <c r="H30" s="17"/>
+      <c r="I30" s="17"/>
+      <c r="J30" s="17"/>
+      <c r="K30" s="17"/>
+      <c r="L30" s="17"/>
+      <c r="M30" s="17"/>
+      <c r="N30" s="17"/>
+      <c r="O30" s="17"/>
+      <c r="P30" s="17"/>
+      <c r="Q30" s="17"/>
+      <c r="R30" s="17"/>
+      <c r="S30" s="17"/>
+      <c r="T30" s="17"/>
+      <c r="U30" s="17"/>
+      <c r="V30" s="17"/>
+      <c r="W30" s="17"/>
+      <c r="X30" s="17"/>
+      <c r="Y30" s="17"/>
+      <c r="Z30" s="17"/>
+      <c r="AA30" s="17"/>
+      <c r="AB30" s="17"/>
+      <c r="AC30" s="17"/>
+      <c r="AD30" s="17"/>
+      <c r="AE30" s="17"/>
+      <c r="AF30" s="17"/>
+      <c r="AG30" s="17"/>
+      <c r="AH30" s="17"/>
+      <c r="AI30" s="17"/>
+      <c r="AJ30" s="17"/>
+      <c r="AK30" s="17"/>
+      <c r="AL30" s="17"/>
+      <c r="AM30" s="17"/>
+      <c r="AN30" s="17"/>
+      <c r="AO30" s="17"/>
+      <c r="AP30" s="17"/>
+      <c r="AQ30" s="17"/>
+      <c r="AR30" s="17"/>
+      <c r="AS30" s="17"/>
+      <c r="AT30" s="17"/>
+      <c r="AU30" s="17"/>
+      <c r="AV30" s="17"/>
+      <c r="AW30" s="17"/>
+      <c r="AX30" s="17"/>
+      <c r="AY30" s="17"/>
+      <c r="AZ30" s="17"/>
+      <c r="BA30" s="17"/>
+      <c r="BB30" s="17"/>
+      <c r="BC30" s="17"/>
+      <c r="BD30" s="17"/>
+      <c r="BE30" s="17"/>
     </row>
     <row r="32" spans="1:57" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -3608,23 +3608,23 @@
       <c r="BD57" s="12"/>
       <c r="BE57" s="12"/>
       <c r="BG57" s="2">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="BH57" s="2">
-        <v>48</v>
+        <v>2</v>
       </c>
       <c r="BI57" s="2">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="BJ57" s="2">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="BK57" s="2">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="BL57" s="2">
         <f>AVERAGE(BG57:BK57)</f>
-        <v>40</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58" spans="1:64" x14ac:dyDescent="0.25">
@@ -3635,7 +3635,7 @@
       <c r="C58" s="12"/>
       <c r="D58" s="12"/>
       <c r="E58" s="12"/>
-      <c r="F58" s="20" t="s">
+      <c r="F58" s="16" t="s">
         <v>46</v>
       </c>
       <c r="G58" s="4"/>
@@ -3814,27 +3814,47 @@
       <c r="BD60" s="6"/>
       <c r="BE60" s="6"/>
       <c r="BG60" s="2">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="BH60" s="2">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="BI60" s="2">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="BJ60" s="2">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="BK60" s="2">
         <v>55</v>
       </c>
       <c r="BL60" s="2">
         <f>AVERAGE(BG60:BK60)</f>
-        <v>40</v>
+        <v>39.200000000000003</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="36">
+    <mergeCell ref="AF12:AN12"/>
+    <mergeCell ref="AF13:AN13"/>
+    <mergeCell ref="AF14:AN14"/>
+    <mergeCell ref="W8:AE8"/>
+    <mergeCell ref="W10:AE10"/>
+    <mergeCell ref="W11:AE11"/>
+    <mergeCell ref="W12:AE12"/>
+    <mergeCell ref="B18:BE20"/>
+    <mergeCell ref="B4:V4"/>
+    <mergeCell ref="W4:AE4"/>
+    <mergeCell ref="AF4:AN4"/>
+    <mergeCell ref="W13:AE13"/>
+    <mergeCell ref="W14:AE14"/>
+    <mergeCell ref="AF5:AN5"/>
+    <mergeCell ref="AF6:AN6"/>
+    <mergeCell ref="AF7:AN7"/>
+    <mergeCell ref="AF8:AN8"/>
+    <mergeCell ref="AF9:AN9"/>
+    <mergeCell ref="AF10:AN10"/>
+    <mergeCell ref="AF11:AN11"/>
     <mergeCell ref="B23:BE25"/>
     <mergeCell ref="B28:BE30"/>
     <mergeCell ref="B5:V5"/>
@@ -3851,26 +3871,6 @@
     <mergeCell ref="W6:AE6"/>
     <mergeCell ref="W7:AE7"/>
     <mergeCell ref="W9:AE9"/>
-    <mergeCell ref="W10:AE10"/>
-    <mergeCell ref="W11:AE11"/>
-    <mergeCell ref="W12:AE12"/>
-    <mergeCell ref="B18:BE20"/>
-    <mergeCell ref="B4:V4"/>
-    <mergeCell ref="W4:AE4"/>
-    <mergeCell ref="AF4:AN4"/>
-    <mergeCell ref="W13:AE13"/>
-    <mergeCell ref="W14:AE14"/>
-    <mergeCell ref="AF5:AN5"/>
-    <mergeCell ref="AF6:AN6"/>
-    <mergeCell ref="AF7:AN7"/>
-    <mergeCell ref="AF8:AN8"/>
-    <mergeCell ref="AF9:AN9"/>
-    <mergeCell ref="AF10:AN10"/>
-    <mergeCell ref="AF11:AN11"/>
-    <mergeCell ref="AF12:AN12"/>
-    <mergeCell ref="AF13:AN13"/>
-    <mergeCell ref="AF14:AN14"/>
-    <mergeCell ref="W8:AE8"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>